<commit_message>
usertest logic + error corrected
</commit_message>
<xml_diff>
--- a/data/Usertest.xlsx
+++ b/data/Usertest.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">timezon</t>
   </si>
   <si>
-    <t xml:space="preserve">Europe/Paris</t>
+    <t xml:space="preserve">Europe/London</t>
   </si>
   <si>
     <t xml:space="preserve">location</t>
@@ -85,27 +85,6 @@
   </si>
   <si>
     <t xml:space="preserve">after</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delete</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Children / teens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insert1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service d0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service after d0</t>
   </si>
 </sst>
 </file>
@@ -340,7 +319,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>1396</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -444,7 +423,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="13.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -457,67 +436,33 @@
       <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>23</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>27</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="C6" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>